<commit_message>
Clean project commit without secrets
</commit_message>
<xml_diff>
--- a/Tracker.xlsx
+++ b/Tracker.xlsx
@@ -40,7 +40,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -67,8 +67,56 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFBFBFBF"/>
         <bgColor rgb="FFBFBFBF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF92D050"/>
       </patternFill>
     </fill>
     <fill>
@@ -126,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -134,9 +182,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1601,42 +1657,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:Q43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="26.6328125" customWidth="1" min="1" max="1"/>
     <col width="27.54296875" customWidth="1" min="2" max="2"/>
-    <col width="14.7265625" customWidth="1" min="3" max="3"/>
-    <col width="16.1796875" customWidth="1" min="4" max="4"/>
+    <col width="16.1796875" customWidth="1" min="3" max="3"/>
+    <col width="15.6328125" customWidth="1" min="4" max="4"/>
+    <col width="15.90625" customWidth="1" min="5" max="5"/>
+    <col width="14.81640625" customWidth="1" min="6" max="6"/>
+    <col width="20.36328125" customWidth="1" min="7" max="7"/>
+    <col width="12.7265625" customWidth="1" min="8" max="8"/>
+    <col width="18.1796875" customWidth="1" min="9" max="9"/>
+    <col width="16.453125" customWidth="1" min="10" max="10"/>
+    <col width="16.36328125" customWidth="1" min="11" max="11"/>
+    <col width="24.81640625" customWidth="1" min="12" max="12"/>
+    <col width="21.6328125" customWidth="1" min="13" max="13"/>
+    <col width="15.7265625" customWidth="1" min="14" max="14"/>
+    <col width="15.453125" customWidth="1" min="15" max="15"/>
+    <col width="23.90625" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.5" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="16" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="G1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="H1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="I1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="J1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="K1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="L1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="M1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="N1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="O1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="P1" s="16" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="Q1" s="16" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -1648,16 +1771,11 @@
           <t>101588348</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Oindrila Chakraborty</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1668,7 +1786,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1678,16 +1851,11 @@
           <t>101582442</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Subhabrata Sengupta</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1698,7 +1866,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1708,16 +1931,11 @@
           <t>101578754</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Ishita Banerjee</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1728,7 +1946,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1738,16 +2011,11 @@
           <t>101560676</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>REDDI KEERTHI</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1758,7 +2026,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1768,16 +2091,11 @@
           <t>101560510</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Anik Tanzim</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1788,8 +2106,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>0</v>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O6" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -1798,28 +2171,78 @@
           <t>101560450</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Anusree Roy</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1828,16 +2251,11 @@
           <t>101560255</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Kumari Ritul</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1848,7 +2266,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1858,16 +2331,11 @@
           <t>101453747</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Moupriya Ganguly</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1878,7 +2346,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1888,16 +2411,11 @@
           <t>101442923</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Ayantik Das</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1908,8 +2426,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>0</v>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L10" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O10" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P10" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -1918,16 +2491,11 @@
           <t>101442680</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Ratul Ghosh</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1938,8 +2506,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>0</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1948,16 +2571,11 @@
           <t>101442606</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Avisake Chowdhury</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1968,8 +2586,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>0</v>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1978,16 +2651,11 @@
           <t>101442577</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Banavathu Naik</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>NA</t>
@@ -1998,7 +2666,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2008,16 +2731,11 @@
           <t>101442457</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Piyush Deb</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2028,7 +2746,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2038,16 +2811,11 @@
           <t>101442398</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Shreya Singh</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2058,7 +2826,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2068,16 +2891,11 @@
           <t>101408941</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Riya Biswas</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2088,7 +2906,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2098,16 +2971,11 @@
           <t>101282639</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Soumya Mondal</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2118,8 +2986,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>0</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -2128,16 +3051,11 @@
           <t>101259073</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Sayanti Pal</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2148,7 +3066,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2158,16 +3131,11 @@
           <t>101148869</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Arunabha Mitra</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2178,7 +3146,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2188,16 +3211,11 @@
           <t>101110378</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Solanki Kundu</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2208,7 +3226,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2218,16 +3291,11 @@
           <t>101744590</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Sunirmal Bera</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2238,8 +3306,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>0</v>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M21" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N21" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -2248,17 +3371,12 @@
           <t>101758893</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Ankita Chhetry</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
@@ -2268,8 +3386,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>1</v>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K22" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O22" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P22" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="23">
@@ -2278,28 +3451,78 @@
           <t>101675169</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Vikash Kumar</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>2</v>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="K23" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L23" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="M23" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N23" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="O23" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -2308,28 +3531,78 @@
           <t>101743106</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Rishagny Choudhury</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>1</v>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L24" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="M24" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P24" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="25">
@@ -2338,16 +3611,11 @@
           <t>101777658</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Kaustav Chakraborty</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2358,8 +3626,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>0</v>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K25" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M25" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N25" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="O25" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P25" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="26">
@@ -2368,28 +3691,78 @@
           <t>101774195</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Deborshi Som</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>1</v>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K26" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L26" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O26" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P26" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -2398,28 +3771,78 @@
           <t>101779334</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>SAQLAIN Mustafa</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>1</v>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I27" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K27" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O27" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P27" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -2428,16 +3851,11 @@
           <t>100682010</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Nazia Afreen</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2448,8 +3866,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>0</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -2458,16 +3931,11 @@
           <t>101752092</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Madhu Komera</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2478,7 +3946,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2488,16 +4011,11 @@
           <t>101675381</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Venkatesh Ulla</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2508,8 +4026,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>0</v>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q30" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -2518,16 +4091,11 @@
           <t>101786698</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>N Jyotheeswar</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2538,8 +4106,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>0</v>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L31" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="M31" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N31" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="O31" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q31" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="32">
@@ -2548,16 +4171,11 @@
           <t>101699107</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>ANKIT Mahali</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2568,8 +4186,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>0</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q32" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -2578,16 +4251,11 @@
           <t>101264925</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Ritwik Acharya</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2598,8 +4266,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>0</v>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M33" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q33" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -2608,28 +4331,78 @@
           <t>101675401</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Abhinav Baranwal</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>1</v>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M34" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O34" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P34" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q34" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="35">
@@ -2638,17 +4411,12 @@
           <t>101755619</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Mukul Kumar</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
@@ -2658,8 +4426,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>1</v>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O35" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q35" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -2668,28 +4491,78 @@
           <t>101675341</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Abhinandan Roy</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>1</v>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="H36" s="10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J36" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="K36" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L36" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="M36" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N36" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="O36" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P36" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q36" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="37">
@@ -2698,28 +4571,78 @@
           <t>101787312</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>ISHWAR Jha</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>1</v>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I37" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O37" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P37" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q37" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="38">
@@ -2728,16 +4651,11 @@
           <t>101775278</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Vivek Nayak</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2748,8 +4666,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>0</v>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L38" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="M38" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O38" s="15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="P38" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q38" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="39">
@@ -2758,16 +4731,11 @@
           <t>101082599</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Aditi Khaitan</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D39" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2778,7 +4746,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F39" t="n">
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2788,17 +4811,12 @@
           <t>101807073</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Sumit Shaw</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
@@ -2808,8 +4826,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F40" t="n">
-        <v>1</v>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H40" s="10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J40" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="K40" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M40" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N40" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P40" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q40" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="41">
@@ -2818,28 +4891,78 @@
           <t>101790824</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Debojyoti Saha</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="E41" s="9" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="F41" t="n">
-        <v>2</v>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J41" s="12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P41" s="17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="Q41" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="42">
@@ -2848,16 +4971,11 @@
           <t>101805990</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Gourab Das</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2868,7 +4986,62 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F42" t="n">
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2878,16 +5051,11 @@
           <t>101676413</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Tushti Thakur</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>NA</t>
@@ -2898,8 +5066,63 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>0</v>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="I43" s="11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="M43" s="13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Q43" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>